<commit_message>
added visuals in a local webpage
</commit_message>
<xml_diff>
--- a/Vouchers/CostSheet.xlsx
+++ b/Vouchers/CostSheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Workspace\Project A7\Vouchers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Education\Workspace\Project A7\Vouchers\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D95937FA-FC5F-4E91-8FDD-D0130A2D27E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3422739B-D769-49E3-A8BF-8B17B6BD9DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="16305" xr2:uid="{FC7D7B7B-0301-4E2A-8B41-42FF0B0D22BF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{FC7D7B7B-0301-4E2A-8B41-42FF0B0D22BF}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>26/06/2026</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>30/07/26</t>
+  </si>
+  <si>
+    <t>28/08/2026</t>
   </si>
 </sst>
 </file>
@@ -480,6 +483,9 @@
       <c r="J5" s="1">
         <v>46030</v>
       </c>
+      <c r="K5" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
@@ -494,9 +500,12 @@
       <c r="H6">
         <v>400</v>
       </c>
+      <c r="K6">
+        <v>2605</v>
+      </c>
       <c r="T6">
         <f>SUM(C6:S6)</f>
-        <v>8610</v>
+        <v>11215</v>
       </c>
     </row>
     <row r="7" spans="2:20" x14ac:dyDescent="0.25">
@@ -519,9 +528,12 @@
         <f>55+20</f>
         <v>75</v>
       </c>
+      <c r="K7">
+        <v>2000</v>
+      </c>
       <c r="T7">
         <f t="shared" ref="T7:T9" si="0">SUM(C7:S7)</f>
-        <v>8625</v>
+        <v>10625</v>
       </c>
     </row>
     <row r="8" spans="2:20" x14ac:dyDescent="0.25">
@@ -543,9 +555,12 @@
       <c r="J8">
         <v>50</v>
       </c>
+      <c r="K8">
+        <v>2000</v>
+      </c>
       <c r="T8">
         <f t="shared" si="0"/>
-        <v>7670</v>
+        <v>9670</v>
       </c>
     </row>
     <row r="9" spans="2:20" x14ac:dyDescent="0.25">
@@ -567,15 +582,18 @@
       <c r="J9">
         <v>320</v>
       </c>
+      <c r="K9">
+        <v>2100</v>
+      </c>
       <c r="T9">
         <f t="shared" si="0"/>
-        <v>7660</v>
+        <v>9760</v>
       </c>
     </row>
     <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="T12" s="2">
         <f>SUM(T6:T9)</f>
-        <v>32565</v>
+        <v>41270</v>
       </c>
     </row>
   </sheetData>

</xml_diff>